<commit_message>
chore: update binary files for token save and export format
</commit_message>
<xml_diff>
--- a/docs/export-format/FM-DC-04 Rev.02 ทะเบียนรายชื่อเอกสารควบคุม Master List.xlsx
+++ b/docs/export-format/FM-DC-04 Rev.02 ทะเบียนรายชื่อเอกสารควบคุม Master List.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365180F5-1099-49D0-8686-C0A4DB93333C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Master List" state="visible" r:id="rId4"/>
+    <sheet name="Master List" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>ทะเบียนรายชื่อเอกสารควบคุม (Master List)</t>
   </si>
   <si>
-    <t>FM-DC-04 Rev.02</t>
-  </si>
-  <si>
     <t>วันที่ปรับปรุง:</t>
   </si>
   <si>
@@ -73,7 +74,7 @@
     <t>QC</t>
   </si>
   <si>
-    <t xml:space="preserve">QC
+    <t>QC
 Lab</t>
   </si>
   <si>
@@ -101,24 +102,24 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Tahoma"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FF0F1059"/>
-      <sz val="16"/>
       <name val="Tahoma"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF666666"/>
-      <sz val="10"/>
       <name val="Tahoma"/>
     </font>
     <font>
@@ -132,8 +133,8 @@
     </font>
     <font>
       <b/>
+      <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
       <name val="Tahoma"/>
     </font>
   </fonts>
@@ -177,16 +178,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -528,9 +532,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -542,148 +546,146 @@
     <col min="8" max="26" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:26" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+      <c r="X2" s="5"/>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="5"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2"/>
-      <c r="Z2" s="2"/>
+      <c r="C4" s="2"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+    <row r="7" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="7" ht="30" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="6"/>
+      <c r="D7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="J7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="K7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="P7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P7" s="5" t="s">
+      <c r="Q7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="Q7" s="5" t="s">
+      <c r="R7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="S7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="T7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="T7" s="5" t="s">
+      <c r="U7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="U7" s="5" t="s">
+      <c r="V7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="V7" s="5" t="s">
+      <c r="W7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="W7" s="5" t="s">
+      <c r="X7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="X7" s="5" t="s">
+      <c r="Y7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Y7" s="5" t="s">
+      <c r="Z7" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -693,6 +695,6 @@
     <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>